<commit_message>
Refine schedule page rendering and sample data
Groups events under a per-date section heading (new groupEventsByDate.ts)
instead of repeating the date on every card, and tightens sample data to
a realistic 3-day/8-event window while keeping date/time format
diversity for the parser tests.

Cards are now dividers/alternating rows instead of boxes. In landscape,
time/location/description lay out as columns that stay vertically
aligned across every card via CSS Subgrid (the <ul> owns the shared
column tracks, each card spans them), with content-sized (not
fixed-width) columns and a Playwright test guarding against the
horizontal-overflow regression a fixed-width floor would reintroduce on
a narrow-but-landscape window.

Amends docs/design/schedule-page.md's Layout design and Breakpoint
strategy decisions to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/event-schedule.xlsx
+++ b/data/event-schedule.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>6:00 PM - 7:30 PM</t>
+    <t>10:00 - 11:00am</t>
   </si>
   <si>
     <t>Studio A</t>
@@ -34,52 +34,61 @@
     <t>Beginner Salsa</t>
   </si>
   <si>
-    <t>8/22/2026</t>
-  </si>
-  <si>
-    <t>6:00pm-7:00pm</t>
+    <t>8/15/2026</t>
+  </si>
+  <si>
+    <t>11:15 - 12:15pm</t>
+  </si>
+  <si>
+    <t>Intermediate Salsa</t>
+  </si>
+  <si>
+    <t>13:00 - 14:00</t>
   </si>
   <si>
     <t>Studio B</t>
   </si>
   <si>
-    <t>Intermediate Salsa</t>
-  </si>
-  <si>
-    <t>August 29, 2026</t>
+    <t>Bachata Basics</t>
+  </si>
+  <si>
+    <t>7 to 8:30pm</t>
+  </si>
+  <si>
+    <t>Salsa Social</t>
+  </si>
+  <si>
+    <t>8/16/2026</t>
+  </si>
+  <si>
+    <t>2:00 - 3:30pm</t>
+  </si>
+  <si>
+    <t>Studio C</t>
+  </si>
+  <si>
+    <t>Cha Cha Workshop</t>
+  </si>
+  <si>
+    <t>9:00 - 10:00</t>
+  </si>
+  <si>
+    <t>Morning Stretch &amp; Salsa Basics</t>
+  </si>
+  <si>
+    <t>August 17, 2026</t>
   </si>
   <si>
     <t>11 - 1pm</t>
   </si>
   <si>
-    <t>Advanced Salsa Workshop</t>
-  </si>
-  <si>
-    <t>9/5/26</t>
-  </si>
-  <si>
-    <t>18:00 - 19:30</t>
-  </si>
-  <si>
-    <t>Studio C</t>
+    <t>Advanced Workshop</t>
+  </si>
+  <si>
+    <t>6:00 p.m. - 7:30 p.m.</t>
   </si>
   <si>
     <t>Bachata Night</t>
-  </si>
-  <si>
-    <t>7 to 8:30pm</t>
-  </si>
-  <si>
-    <t>Salsa Social</t>
-  </si>
-  <si>
-    <t>2026-09-19</t>
-  </si>
-  <si>
-    <t>6:00 p.m. - 7:30 p.m.</t>
-  </si>
-  <si>
-    <t>Cha Cha Basics</t>
   </si>
 </sst>
 </file>
@@ -460,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -499,66 +508,94 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="D5" t="s">
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>46277</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46251</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="B8" t="s">
         <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>